<commit_message>
Extended BAU model functionality and improved backend formula handling
- Updated BAU upload template to include tariff, demand, upstream cost, CAPEX, OPEX, and D&A, allowing comparison with other models.

- Added "Technoeconomic Inputs" section and CAPEX calculation view for BAU in the platform, alongside the carbon credits section.

- Refactored backend (main.py, Uvicorn) to support new BAU data structure.

- Improved ExcelFormulaEngine: fixed dictionary key expansion logic to correctly substitute repeated {fuel} or {fuels} tokens, increasing robustness and consistency.

- Advanced backend formula development in formulas_map.json.
</commit_message>
<xml_diff>
--- a/backend/{templates}/upload-bau.xlsx
+++ b/backend/{templates}/upload-bau.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8954da175e61d5af/Escritorio/IIT/CC-WBT/backend/{templates}/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="30" documentId="6_{A60EB3FB-659D-4A85-93E3-E4EBBB4CC8A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BBD75CD8-82CE-4F25-AEFE-ADCCD66BC085}"/>
+  <xr:revisionPtr revIDLastSave="32" documentId="6_{A60EB3FB-659D-4A85-93E3-E4EBBB4CC8A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A7AED5CE-0320-4B89-B8EC-20A24266791A}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="11370" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Carbon Credits" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="30">
   <si>
     <t>Units</t>
   </si>
@@ -85,13 +85,49 @@
     <t>Demand - OFF-GRID</t>
   </si>
   <si>
-    <t xml:space="preserve">- </t>
+    <t>Outputs - GRID</t>
   </si>
   <si>
-    <t>GRID</t>
+    <t>-</t>
   </si>
   <si>
-    <t>OFF-GRID</t>
+    <t>CAPEX - GRID</t>
+  </si>
+  <si>
+    <t>M$</t>
+  </si>
+  <si>
+    <t>OPEX - GRID</t>
+  </si>
+  <si>
+    <t>D&amp;A - GRID</t>
+  </si>
+  <si>
+    <t>years</t>
+  </si>
+  <si>
+    <t>Outputs - OFF-GRID</t>
+  </si>
+  <si>
+    <t>CAPEX - OFF-GRID</t>
+  </si>
+  <si>
+    <t>OPEX - OFF-GRID</t>
+  </si>
+  <si>
+    <t>D&amp;A - OFF-GRID</t>
+  </si>
+  <si>
+    <t>Outputs</t>
+  </si>
+  <si>
+    <t>CAPEX</t>
+  </si>
+  <si>
+    <t>OPEX</t>
+  </si>
+  <si>
+    <t>D&amp;A</t>
   </si>
 </sst>
 </file>
@@ -149,7 +185,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -177,6 +213,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -209,7 +251,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -241,12 +283,27 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" xfId="1" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="3" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="3" fontId="5" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="3" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -264,6 +321,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -809,7 +870,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{243625B2-4F16-4A46-A9C0-68EF42D0E994}">
-  <dimension ref="A1:AQ8"/>
+  <dimension ref="A1:AQ14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="26.26953125" customWidth="1"/>
@@ -948,141 +1009,141 @@
     </row>
     <row r="2" spans="1:43" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A2" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="B2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="D2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="E2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="F2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="G2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="H2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="I2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="J2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="K2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="L2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="M2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="N2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="O2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="P2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="R2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="S2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="T2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="U2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="V2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="W2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="X2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="Y2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="Z2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="AA2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="AB2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="AC2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="AD2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="AE2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="AF2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="AG2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="AH2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="AI2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="AJ2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="AK2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="AL2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="AM2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="AN2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="AO2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="AP2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="AQ2" s="12" t="s">
-        <v>15</v>
+        <v>10</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="6">
+        <v>0</v>
+      </c>
+      <c r="D2" s="6">
+        <v>0</v>
+      </c>
+      <c r="E2" s="6">
+        <v>0</v>
+      </c>
+      <c r="F2" s="6">
+        <v>0</v>
+      </c>
+      <c r="G2" s="6">
+        <v>0</v>
+      </c>
+      <c r="H2" s="6">
+        <v>0</v>
+      </c>
+      <c r="I2" s="6">
+        <v>0</v>
+      </c>
+      <c r="J2" s="6">
+        <v>0</v>
+      </c>
+      <c r="K2" s="6">
+        <v>0</v>
+      </c>
+      <c r="L2" s="6">
+        <v>0</v>
+      </c>
+      <c r="M2" s="6">
+        <v>0</v>
+      </c>
+      <c r="N2" s="6">
+        <v>0</v>
+      </c>
+      <c r="O2" s="6">
+        <v>0</v>
+      </c>
+      <c r="P2" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="6">
+        <v>0</v>
+      </c>
+      <c r="R2" s="6">
+        <v>0</v>
+      </c>
+      <c r="S2" s="6">
+        <v>0</v>
+      </c>
+      <c r="T2" s="6">
+        <v>0</v>
+      </c>
+      <c r="U2" s="6">
+        <v>0</v>
+      </c>
+      <c r="V2" s="6">
+        <v>0</v>
+      </c>
+      <c r="W2" s="6">
+        <v>0</v>
+      </c>
+      <c r="X2" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y2" s="6">
+        <v>0</v>
+      </c>
+      <c r="Z2" s="6">
+        <v>0</v>
+      </c>
+      <c r="AA2" s="6">
+        <v>0</v>
+      </c>
+      <c r="AB2" s="6">
+        <v>0</v>
+      </c>
+      <c r="AC2" s="6">
+        <v>0</v>
+      </c>
+      <c r="AD2" s="6">
+        <v>0</v>
+      </c>
+      <c r="AE2" s="6">
+        <v>0</v>
+      </c>
+      <c r="AF2" s="6">
+        <v>0</v>
+      </c>
+      <c r="AG2" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH2" s="6">
+        <v>0</v>
+      </c>
+      <c r="AI2" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ2" s="6">
+        <v>0</v>
+      </c>
+      <c r="AK2" s="6">
+        <v>0</v>
+      </c>
+      <c r="AL2" s="6">
+        <v>0</v>
+      </c>
+      <c r="AM2" s="6">
+        <v>0</v>
+      </c>
+      <c r="AN2" s="6">
+        <v>0</v>
+      </c>
+      <c r="AO2" s="6">
+        <v>0</v>
+      </c>
+      <c r="AP2" s="6">
+        <v>0</v>
+      </c>
+      <c r="AQ2" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:43" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="13" t="s">
-        <v>10</v>
+      <c r="A3" s="7" t="s">
+        <v>11</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C3" s="6">
         <v>0</v>
@@ -1209,11 +1270,11 @@
       </c>
     </row>
     <row r="4" spans="1:43" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="13" t="s">
-        <v>11</v>
+      <c r="A4" s="7" t="s">
+        <v>12</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C4" s="6">
         <v>0</v>
@@ -1340,273 +1401,273 @@
       </c>
     </row>
     <row r="5" spans="1:43" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="13" t="s">
-        <v>12</v>
+      <c r="A5" s="12" t="s">
+        <v>15</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" s="6">
-        <v>0</v>
-      </c>
-      <c r="D5" s="6">
-        <v>0</v>
-      </c>
-      <c r="E5" s="6">
-        <v>0</v>
-      </c>
-      <c r="F5" s="6">
-        <v>0</v>
-      </c>
-      <c r="G5" s="6">
-        <v>0</v>
-      </c>
-      <c r="H5" s="6">
-        <v>0</v>
-      </c>
-      <c r="I5" s="6">
-        <v>0</v>
-      </c>
-      <c r="J5" s="6">
-        <v>0</v>
-      </c>
-      <c r="K5" s="6">
-        <v>0</v>
-      </c>
-      <c r="L5" s="6">
-        <v>0</v>
-      </c>
-      <c r="M5" s="6">
-        <v>0</v>
-      </c>
-      <c r="N5" s="6">
-        <v>0</v>
-      </c>
-      <c r="O5" s="6">
-        <v>0</v>
-      </c>
-      <c r="P5" s="6">
-        <v>0</v>
-      </c>
-      <c r="Q5" s="6">
-        <v>0</v>
-      </c>
-      <c r="R5" s="6">
-        <v>0</v>
-      </c>
-      <c r="S5" s="6">
-        <v>0</v>
-      </c>
-      <c r="T5" s="6">
-        <v>0</v>
-      </c>
-      <c r="U5" s="6">
-        <v>0</v>
-      </c>
-      <c r="V5" s="6">
-        <v>0</v>
-      </c>
-      <c r="W5" s="6">
-        <v>0</v>
-      </c>
-      <c r="X5" s="6">
-        <v>0</v>
-      </c>
-      <c r="Y5" s="6">
-        <v>0</v>
-      </c>
-      <c r="Z5" s="6">
-        <v>0</v>
-      </c>
-      <c r="AA5" s="6">
-        <v>0</v>
-      </c>
-      <c r="AB5" s="6">
-        <v>0</v>
-      </c>
-      <c r="AC5" s="6">
-        <v>0</v>
-      </c>
-      <c r="AD5" s="6">
-        <v>0</v>
-      </c>
-      <c r="AE5" s="6">
-        <v>0</v>
-      </c>
-      <c r="AF5" s="6">
-        <v>0</v>
-      </c>
-      <c r="AG5" s="6">
-        <v>0</v>
-      </c>
-      <c r="AH5" s="6">
-        <v>0</v>
-      </c>
-      <c r="AI5" s="6">
-        <v>0</v>
-      </c>
-      <c r="AJ5" s="6">
-        <v>0</v>
-      </c>
-      <c r="AK5" s="6">
-        <v>0</v>
-      </c>
-      <c r="AL5" s="6">
-        <v>0</v>
-      </c>
-      <c r="AM5" s="6">
-        <v>0</v>
-      </c>
-      <c r="AN5" s="6">
-        <v>0</v>
-      </c>
-      <c r="AO5" s="6">
-        <v>0</v>
-      </c>
-      <c r="AP5" s="6">
-        <v>0</v>
-      </c>
-      <c r="AQ5" s="6">
-        <v>0</v>
+        <v>16</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="H5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="I5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="J5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="K5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="L5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="M5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="N5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="O5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="P5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="R5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="S5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="T5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="U5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="V5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="W5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="X5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="Y5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="Z5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AA5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AB5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AC5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AD5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AE5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AF5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AH5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AI5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AJ5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AK5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AL5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AM5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AN5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AO5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AP5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AQ5" s="9" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:43" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="D6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="E6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="F6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="G6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="H6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="I6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="J6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="K6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="L6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="M6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="N6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="O6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="P6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="R6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="S6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="T6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="U6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="V6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="W6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="X6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="Y6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="Z6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="AA6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="AB6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="AC6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="AD6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="AE6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="AF6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="AG6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="AH6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="AI6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="AJ6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="AK6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="AL6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="AM6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="AN6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="AO6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="AP6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="AQ6" s="12" t="s">
-        <v>15</v>
+      <c r="B6" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="6">
+        <v>0</v>
+      </c>
+      <c r="D6" s="6">
+        <v>0</v>
+      </c>
+      <c r="E6" s="6">
+        <v>0</v>
+      </c>
+      <c r="F6" s="6">
+        <v>0</v>
+      </c>
+      <c r="G6" s="6">
+        <v>0</v>
+      </c>
+      <c r="H6" s="6">
+        <v>0</v>
+      </c>
+      <c r="I6" s="6">
+        <v>0</v>
+      </c>
+      <c r="J6" s="6">
+        <v>0</v>
+      </c>
+      <c r="K6" s="6">
+        <v>0</v>
+      </c>
+      <c r="L6" s="6">
+        <v>0</v>
+      </c>
+      <c r="M6" s="6">
+        <v>0</v>
+      </c>
+      <c r="N6" s="6">
+        <v>0</v>
+      </c>
+      <c r="O6" s="6">
+        <v>0</v>
+      </c>
+      <c r="P6" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="6">
+        <v>0</v>
+      </c>
+      <c r="R6" s="6">
+        <v>0</v>
+      </c>
+      <c r="S6" s="6">
+        <v>0</v>
+      </c>
+      <c r="T6" s="6">
+        <v>0</v>
+      </c>
+      <c r="U6" s="6">
+        <v>0</v>
+      </c>
+      <c r="V6" s="6">
+        <v>0</v>
+      </c>
+      <c r="W6" s="6">
+        <v>0</v>
+      </c>
+      <c r="X6" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y6" s="6">
+        <v>0</v>
+      </c>
+      <c r="Z6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AA6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AB6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AC6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AD6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AE6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AF6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AG6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AI6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AK6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AL6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AM6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AN6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AO6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AP6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AQ6" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:43" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="13" t="s">
-        <v>13</v>
+      <c r="A7" s="14" t="s">
+        <v>19</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="C7" s="6">
         <v>0</v>
@@ -1733,134 +1794,920 @@
       </c>
     </row>
     <row r="8" spans="1:43" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A8" s="13" t="s">
+      <c r="A8" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="16">
+        <v>0</v>
+      </c>
+      <c r="D8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="E8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="G8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="H8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="I8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="J8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="K8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="L8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="M8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="N8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="O8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="P8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="R8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="S8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="T8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="U8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="V8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="W8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="X8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="Y8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="Z8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AA8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AB8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AC8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AD8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AE8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AF8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AH8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AI8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AJ8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AK8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AL8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AM8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AN8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AO8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AP8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AQ8" s="16" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:43" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A9" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="6">
+        <v>0</v>
+      </c>
+      <c r="D9" s="6">
+        <v>0</v>
+      </c>
+      <c r="E9" s="6">
+        <v>0</v>
+      </c>
+      <c r="F9" s="6">
+        <v>0</v>
+      </c>
+      <c r="G9" s="6">
+        <v>0</v>
+      </c>
+      <c r="H9" s="6">
+        <v>0</v>
+      </c>
+      <c r="I9" s="6">
+        <v>0</v>
+      </c>
+      <c r="J9" s="6">
+        <v>0</v>
+      </c>
+      <c r="K9" s="6">
+        <v>0</v>
+      </c>
+      <c r="L9" s="6">
+        <v>0</v>
+      </c>
+      <c r="M9" s="6">
+        <v>0</v>
+      </c>
+      <c r="N9" s="6">
+        <v>0</v>
+      </c>
+      <c r="O9" s="6">
+        <v>0</v>
+      </c>
+      <c r="P9" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="6">
+        <v>0</v>
+      </c>
+      <c r="R9" s="6">
+        <v>0</v>
+      </c>
+      <c r="S9" s="6">
+        <v>0</v>
+      </c>
+      <c r="T9" s="6">
+        <v>0</v>
+      </c>
+      <c r="U9" s="6">
+        <v>0</v>
+      </c>
+      <c r="V9" s="6">
+        <v>0</v>
+      </c>
+      <c r="W9" s="6">
+        <v>0</v>
+      </c>
+      <c r="X9" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y9" s="6">
+        <v>0</v>
+      </c>
+      <c r="Z9" s="6">
+        <v>0</v>
+      </c>
+      <c r="AA9" s="6">
+        <v>0</v>
+      </c>
+      <c r="AB9" s="6">
+        <v>0</v>
+      </c>
+      <c r="AC9" s="6">
+        <v>0</v>
+      </c>
+      <c r="AD9" s="6">
+        <v>0</v>
+      </c>
+      <c r="AE9" s="6">
+        <v>0</v>
+      </c>
+      <c r="AF9" s="6">
+        <v>0</v>
+      </c>
+      <c r="AG9" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH9" s="6">
+        <v>0</v>
+      </c>
+      <c r="AI9" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ9" s="6">
+        <v>0</v>
+      </c>
+      <c r="AK9" s="6">
+        <v>0</v>
+      </c>
+      <c r="AL9" s="6">
+        <v>0</v>
+      </c>
+      <c r="AM9" s="6">
+        <v>0</v>
+      </c>
+      <c r="AN9" s="6">
+        <v>0</v>
+      </c>
+      <c r="AO9" s="6">
+        <v>0</v>
+      </c>
+      <c r="AP9" s="6">
+        <v>0</v>
+      </c>
+      <c r="AQ9" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:43" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A10" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B10" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="6">
-        <v>0</v>
-      </c>
-      <c r="D8" s="6">
-        <v>0</v>
-      </c>
-      <c r="E8" s="6">
-        <v>0</v>
-      </c>
-      <c r="F8" s="6">
-        <v>0</v>
-      </c>
-      <c r="G8" s="6">
-        <v>0</v>
-      </c>
-      <c r="H8" s="6">
-        <v>0</v>
-      </c>
-      <c r="I8" s="6">
-        <v>0</v>
-      </c>
-      <c r="J8" s="6">
-        <v>0</v>
-      </c>
-      <c r="K8" s="6">
-        <v>0</v>
-      </c>
-      <c r="L8" s="6">
-        <v>0</v>
-      </c>
-      <c r="M8" s="6">
-        <v>0</v>
-      </c>
-      <c r="N8" s="6">
-        <v>0</v>
-      </c>
-      <c r="O8" s="6">
-        <v>0</v>
-      </c>
-      <c r="P8" s="6">
-        <v>0</v>
-      </c>
-      <c r="Q8" s="6">
-        <v>0</v>
-      </c>
-      <c r="R8" s="6">
-        <v>0</v>
-      </c>
-      <c r="S8" s="6">
-        <v>0</v>
-      </c>
-      <c r="T8" s="6">
-        <v>0</v>
-      </c>
-      <c r="U8" s="6">
-        <v>0</v>
-      </c>
-      <c r="V8" s="6">
-        <v>0</v>
-      </c>
-      <c r="W8" s="6">
-        <v>0</v>
-      </c>
-      <c r="X8" s="6">
-        <v>0</v>
-      </c>
-      <c r="Y8" s="6">
-        <v>0</v>
-      </c>
-      <c r="Z8" s="6">
-        <v>0</v>
-      </c>
-      <c r="AA8" s="6">
-        <v>0</v>
-      </c>
-      <c r="AB8" s="6">
-        <v>0</v>
-      </c>
-      <c r="AC8" s="6">
-        <v>0</v>
-      </c>
-      <c r="AD8" s="6">
-        <v>0</v>
-      </c>
-      <c r="AE8" s="6">
-        <v>0</v>
-      </c>
-      <c r="AF8" s="6">
-        <v>0</v>
-      </c>
-      <c r="AG8" s="6">
-        <v>0</v>
-      </c>
-      <c r="AH8" s="6">
-        <v>0</v>
-      </c>
-      <c r="AI8" s="6">
-        <v>0</v>
-      </c>
-      <c r="AJ8" s="6">
-        <v>0</v>
-      </c>
-      <c r="AK8" s="6">
-        <v>0</v>
-      </c>
-      <c r="AL8" s="6">
-        <v>0</v>
-      </c>
-      <c r="AM8" s="6">
-        <v>0</v>
-      </c>
-      <c r="AN8" s="6">
-        <v>0</v>
-      </c>
-      <c r="AO8" s="6">
-        <v>0</v>
-      </c>
-      <c r="AP8" s="6">
-        <v>0</v>
-      </c>
-      <c r="AQ8" s="6">
-        <v>0</v>
+      <c r="C10" s="6">
+        <v>0</v>
+      </c>
+      <c r="D10" s="6">
+        <v>0</v>
+      </c>
+      <c r="E10" s="6">
+        <v>0</v>
+      </c>
+      <c r="F10" s="6">
+        <v>0</v>
+      </c>
+      <c r="G10" s="6">
+        <v>0</v>
+      </c>
+      <c r="H10" s="6">
+        <v>0</v>
+      </c>
+      <c r="I10" s="6">
+        <v>0</v>
+      </c>
+      <c r="J10" s="6">
+        <v>0</v>
+      </c>
+      <c r="K10" s="6">
+        <v>0</v>
+      </c>
+      <c r="L10" s="6">
+        <v>0</v>
+      </c>
+      <c r="M10" s="6">
+        <v>0</v>
+      </c>
+      <c r="N10" s="6">
+        <v>0</v>
+      </c>
+      <c r="O10" s="6">
+        <v>0</v>
+      </c>
+      <c r="P10" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="6">
+        <v>0</v>
+      </c>
+      <c r="R10" s="6">
+        <v>0</v>
+      </c>
+      <c r="S10" s="6">
+        <v>0</v>
+      </c>
+      <c r="T10" s="6">
+        <v>0</v>
+      </c>
+      <c r="U10" s="6">
+        <v>0</v>
+      </c>
+      <c r="V10" s="6">
+        <v>0</v>
+      </c>
+      <c r="W10" s="6">
+        <v>0</v>
+      </c>
+      <c r="X10" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y10" s="6">
+        <v>0</v>
+      </c>
+      <c r="Z10" s="6">
+        <v>0</v>
+      </c>
+      <c r="AA10" s="6">
+        <v>0</v>
+      </c>
+      <c r="AB10" s="6">
+        <v>0</v>
+      </c>
+      <c r="AC10" s="6">
+        <v>0</v>
+      </c>
+      <c r="AD10" s="6">
+        <v>0</v>
+      </c>
+      <c r="AE10" s="6">
+        <v>0</v>
+      </c>
+      <c r="AF10" s="6">
+        <v>0</v>
+      </c>
+      <c r="AG10" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH10" s="6">
+        <v>0</v>
+      </c>
+      <c r="AI10" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ10" s="6">
+        <v>0</v>
+      </c>
+      <c r="AK10" s="6">
+        <v>0</v>
+      </c>
+      <c r="AL10" s="6">
+        <v>0</v>
+      </c>
+      <c r="AM10" s="6">
+        <v>0</v>
+      </c>
+      <c r="AN10" s="6">
+        <v>0</v>
+      </c>
+      <c r="AO10" s="6">
+        <v>0</v>
+      </c>
+      <c r="AP10" s="6">
+        <v>0</v>
+      </c>
+      <c r="AQ10" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:43" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A11" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="H11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="I11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="J11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="K11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="L11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="M11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="N11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="O11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="P11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="R11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="S11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="T11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="U11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="V11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="W11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="X11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="Y11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="Z11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AA11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AB11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AC11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AD11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AE11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AF11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AH11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AI11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AJ11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AK11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AL11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AM11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AN11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AO11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AP11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AQ11" s="9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:43" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A12" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="6">
+        <v>0</v>
+      </c>
+      <c r="D12" s="6">
+        <v>0</v>
+      </c>
+      <c r="E12" s="6">
+        <v>0</v>
+      </c>
+      <c r="F12" s="6">
+        <v>0</v>
+      </c>
+      <c r="G12" s="6">
+        <v>0</v>
+      </c>
+      <c r="H12" s="6">
+        <v>0</v>
+      </c>
+      <c r="I12" s="6">
+        <v>0</v>
+      </c>
+      <c r="J12" s="6">
+        <v>0</v>
+      </c>
+      <c r="K12" s="6">
+        <v>0</v>
+      </c>
+      <c r="L12" s="6">
+        <v>0</v>
+      </c>
+      <c r="M12" s="6">
+        <v>0</v>
+      </c>
+      <c r="N12" s="6">
+        <v>0</v>
+      </c>
+      <c r="O12" s="6">
+        <v>0</v>
+      </c>
+      <c r="P12" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="6">
+        <v>0</v>
+      </c>
+      <c r="R12" s="6">
+        <v>0</v>
+      </c>
+      <c r="S12" s="6">
+        <v>0</v>
+      </c>
+      <c r="T12" s="6">
+        <v>0</v>
+      </c>
+      <c r="U12" s="6">
+        <v>0</v>
+      </c>
+      <c r="V12" s="6">
+        <v>0</v>
+      </c>
+      <c r="W12" s="6">
+        <v>0</v>
+      </c>
+      <c r="X12" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y12" s="6">
+        <v>0</v>
+      </c>
+      <c r="Z12" s="6">
+        <v>0</v>
+      </c>
+      <c r="AA12" s="6">
+        <v>0</v>
+      </c>
+      <c r="AB12" s="6">
+        <v>0</v>
+      </c>
+      <c r="AC12" s="6">
+        <v>0</v>
+      </c>
+      <c r="AD12" s="6">
+        <v>0</v>
+      </c>
+      <c r="AE12" s="6">
+        <v>0</v>
+      </c>
+      <c r="AF12" s="6">
+        <v>0</v>
+      </c>
+      <c r="AG12" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH12" s="6">
+        <v>0</v>
+      </c>
+      <c r="AI12" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ12" s="6">
+        <v>0</v>
+      </c>
+      <c r="AK12" s="6">
+        <v>0</v>
+      </c>
+      <c r="AL12" s="6">
+        <v>0</v>
+      </c>
+      <c r="AM12" s="6">
+        <v>0</v>
+      </c>
+      <c r="AN12" s="6">
+        <v>0</v>
+      </c>
+      <c r="AO12" s="6">
+        <v>0</v>
+      </c>
+      <c r="AP12" s="6">
+        <v>0</v>
+      </c>
+      <c r="AQ12" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:43" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A13" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" s="6">
+        <v>0</v>
+      </c>
+      <c r="D13" s="6">
+        <v>0</v>
+      </c>
+      <c r="E13" s="6">
+        <v>0</v>
+      </c>
+      <c r="F13" s="6">
+        <v>0</v>
+      </c>
+      <c r="G13" s="6">
+        <v>0</v>
+      </c>
+      <c r="H13" s="6">
+        <v>0</v>
+      </c>
+      <c r="I13" s="6">
+        <v>0</v>
+      </c>
+      <c r="J13" s="6">
+        <v>0</v>
+      </c>
+      <c r="K13" s="6">
+        <v>0</v>
+      </c>
+      <c r="L13" s="6">
+        <v>0</v>
+      </c>
+      <c r="M13" s="6">
+        <v>0</v>
+      </c>
+      <c r="N13" s="6">
+        <v>0</v>
+      </c>
+      <c r="O13" s="6">
+        <v>0</v>
+      </c>
+      <c r="P13" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="6">
+        <v>0</v>
+      </c>
+      <c r="R13" s="6">
+        <v>0</v>
+      </c>
+      <c r="S13" s="6">
+        <v>0</v>
+      </c>
+      <c r="T13" s="6">
+        <v>0</v>
+      </c>
+      <c r="U13" s="6">
+        <v>0</v>
+      </c>
+      <c r="V13" s="6">
+        <v>0</v>
+      </c>
+      <c r="W13" s="6">
+        <v>0</v>
+      </c>
+      <c r="X13" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y13" s="6">
+        <v>0</v>
+      </c>
+      <c r="Z13" s="6">
+        <v>0</v>
+      </c>
+      <c r="AA13" s="6">
+        <v>0</v>
+      </c>
+      <c r="AB13" s="6">
+        <v>0</v>
+      </c>
+      <c r="AC13" s="6">
+        <v>0</v>
+      </c>
+      <c r="AD13" s="6">
+        <v>0</v>
+      </c>
+      <c r="AE13" s="6">
+        <v>0</v>
+      </c>
+      <c r="AF13" s="6">
+        <v>0</v>
+      </c>
+      <c r="AG13" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH13" s="6">
+        <v>0</v>
+      </c>
+      <c r="AI13" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ13" s="6">
+        <v>0</v>
+      </c>
+      <c r="AK13" s="6">
+        <v>0</v>
+      </c>
+      <c r="AL13" s="6">
+        <v>0</v>
+      </c>
+      <c r="AM13" s="6">
+        <v>0</v>
+      </c>
+      <c r="AN13" s="6">
+        <v>0</v>
+      </c>
+      <c r="AO13" s="6">
+        <v>0</v>
+      </c>
+      <c r="AP13" s="6">
+        <v>0</v>
+      </c>
+      <c r="AQ13" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:43" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A14" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C14" s="16">
+        <v>0</v>
+      </c>
+      <c r="D14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="E14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="G14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="H14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="I14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="J14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="K14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="L14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="M14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="N14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="O14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="P14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="R14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="S14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="T14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="U14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="V14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="W14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="X14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="Y14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="Z14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AA14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AB14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AC14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AD14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AE14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AF14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AH14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AI14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AJ14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AK14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AL14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AM14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AN14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AO14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AP14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AQ14" s="16" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -1870,7 +2717,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F628CF7D-7E52-48B4-A8ED-0C4CB970313E}">
-  <dimension ref="A1:AQ4"/>
+  <dimension ref="A1:AQ8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:43" ht="15.5" x14ac:dyDescent="0.35">
@@ -2005,7 +2852,7 @@
       </c>
     </row>
     <row r="2" spans="1:43" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="7" t="s">
         <v>5</v>
       </c>
       <c r="B2" s="8" t="s">
@@ -2136,7 +2983,7 @@
       </c>
     </row>
     <row r="3" spans="1:43" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="7" t="s">
         <v>7</v>
       </c>
       <c r="B3" s="8" t="s">
@@ -2267,7 +3114,7 @@
       </c>
     </row>
     <row r="4" spans="1:43" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="7" t="s">
         <v>9</v>
       </c>
       <c r="B4" s="8" t="s">
@@ -2395,6 +3242,530 @@
       </c>
       <c r="AQ4" s="6">
         <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:43" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="H5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="I5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="J5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="K5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="L5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="M5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="N5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="O5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="P5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="R5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="S5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="T5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="U5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="V5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="W5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="X5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="Y5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="Z5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AA5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AB5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AC5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AD5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AE5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AF5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AH5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AI5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AJ5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AK5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AL5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AM5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AN5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AO5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AP5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AQ5" s="9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:43" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A6" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="6">
+        <v>0</v>
+      </c>
+      <c r="D6" s="6">
+        <v>0</v>
+      </c>
+      <c r="E6" s="6">
+        <v>0</v>
+      </c>
+      <c r="F6" s="6">
+        <v>0</v>
+      </c>
+      <c r="G6" s="6">
+        <v>0</v>
+      </c>
+      <c r="H6" s="6">
+        <v>0</v>
+      </c>
+      <c r="I6" s="6">
+        <v>0</v>
+      </c>
+      <c r="J6" s="6">
+        <v>0</v>
+      </c>
+      <c r="K6" s="6">
+        <v>0</v>
+      </c>
+      <c r="L6" s="6">
+        <v>0</v>
+      </c>
+      <c r="M6" s="6">
+        <v>0</v>
+      </c>
+      <c r="N6" s="6">
+        <v>0</v>
+      </c>
+      <c r="O6" s="6">
+        <v>0</v>
+      </c>
+      <c r="P6" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="6">
+        <v>0</v>
+      </c>
+      <c r="R6" s="6">
+        <v>0</v>
+      </c>
+      <c r="S6" s="6">
+        <v>0</v>
+      </c>
+      <c r="T6" s="6">
+        <v>0</v>
+      </c>
+      <c r="U6" s="6">
+        <v>0</v>
+      </c>
+      <c r="V6" s="6">
+        <v>0</v>
+      </c>
+      <c r="W6" s="6">
+        <v>0</v>
+      </c>
+      <c r="X6" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y6" s="6">
+        <v>0</v>
+      </c>
+      <c r="Z6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AA6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AB6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AC6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AD6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AE6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AF6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AG6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AI6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AK6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AL6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AM6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AN6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AO6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AP6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AQ6" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:43" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A7" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="6">
+        <v>0</v>
+      </c>
+      <c r="D7" s="6">
+        <v>0</v>
+      </c>
+      <c r="E7" s="6">
+        <v>0</v>
+      </c>
+      <c r="F7" s="6">
+        <v>0</v>
+      </c>
+      <c r="G7" s="6">
+        <v>0</v>
+      </c>
+      <c r="H7" s="6">
+        <v>0</v>
+      </c>
+      <c r="I7" s="6">
+        <v>0</v>
+      </c>
+      <c r="J7" s="6">
+        <v>0</v>
+      </c>
+      <c r="K7" s="6">
+        <v>0</v>
+      </c>
+      <c r="L7" s="6">
+        <v>0</v>
+      </c>
+      <c r="M7" s="6">
+        <v>0</v>
+      </c>
+      <c r="N7" s="6">
+        <v>0</v>
+      </c>
+      <c r="O7" s="6">
+        <v>0</v>
+      </c>
+      <c r="P7" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="6">
+        <v>0</v>
+      </c>
+      <c r="R7" s="6">
+        <v>0</v>
+      </c>
+      <c r="S7" s="6">
+        <v>0</v>
+      </c>
+      <c r="T7" s="6">
+        <v>0</v>
+      </c>
+      <c r="U7" s="6">
+        <v>0</v>
+      </c>
+      <c r="V7" s="6">
+        <v>0</v>
+      </c>
+      <c r="W7" s="6">
+        <v>0</v>
+      </c>
+      <c r="X7" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y7" s="6">
+        <v>0</v>
+      </c>
+      <c r="Z7" s="6">
+        <v>0</v>
+      </c>
+      <c r="AA7" s="6">
+        <v>0</v>
+      </c>
+      <c r="AB7" s="6">
+        <v>0</v>
+      </c>
+      <c r="AC7" s="6">
+        <v>0</v>
+      </c>
+      <c r="AD7" s="6">
+        <v>0</v>
+      </c>
+      <c r="AE7" s="6">
+        <v>0</v>
+      </c>
+      <c r="AF7" s="6">
+        <v>0</v>
+      </c>
+      <c r="AG7" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH7" s="6">
+        <v>0</v>
+      </c>
+      <c r="AI7" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ7" s="6">
+        <v>0</v>
+      </c>
+      <c r="AK7" s="6">
+        <v>0</v>
+      </c>
+      <c r="AL7" s="6">
+        <v>0</v>
+      </c>
+      <c r="AM7" s="6">
+        <v>0</v>
+      </c>
+      <c r="AN7" s="6">
+        <v>0</v>
+      </c>
+      <c r="AO7" s="6">
+        <v>0</v>
+      </c>
+      <c r="AP7" s="6">
+        <v>0</v>
+      </c>
+      <c r="AQ7" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:43" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A8" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="16">
+        <v>0</v>
+      </c>
+      <c r="D8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="E8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="G8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="H8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="I8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="J8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="K8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="L8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="M8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="N8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="O8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="P8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="R8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="S8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="T8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="U8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="V8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="W8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="X8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="Y8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="Z8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AA8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AB8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AC8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AD8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AE8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AF8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AH8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AI8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AJ8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AK8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AL8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AM8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AN8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AO8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AP8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="AQ8" s="16" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>